<commit_message>
19° Commit- Aggiornamento repo delle patch e dei trattamenti di Core
</commit_message>
<xml_diff>
--- a/patch/docs/patchList_protocolCore.xlsx
+++ b/patch/docs/patchList_protocolCore.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcorbara\Documents\ArgoX3_API_Mobile_CORE\patch\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983A50C2-4D39-4F03-BB65-E29FFB601C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C819E5-5743-46DC-87DD-04629E39D1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core - patchList" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="58">
   <si>
     <t>SRC_X3_V12_X_V1_0</t>
   </si>
@@ -278,24 +278,12 @@
     <t>Controller</t>
   </si>
   <si>
-    <t>N° tabella - X3Cloud</t>
-  </si>
-  <si>
-    <t>N° tabella - Terremerse - SVIL-COLL</t>
-  </si>
-  <si>
-    <t>N° tabella - Piave -SVIL -PROD</t>
-  </si>
-  <si>
     <t>N° tabella - Cloud 2024R2 v12 -PROD</t>
   </si>
   <si>
     <t>N° tabella -EFFORT -TEST</t>
   </si>
   <si>
-    <t>*</t>
-  </si>
-  <si>
     <t>Tabella Diversa - Controller (*Definizione- *Dati)</t>
   </si>
   <si>
@@ -305,13 +293,40 @@
     <t>Abilitazioni Funzionali: dal taso [+] aggiungi le funzioni dell'AppCore AX3M dell'ambiente su cui hai appena installato la patch</t>
   </si>
   <si>
-    <t>6001/6002</t>
-  </si>
-  <si>
     <t>EFFORT -PROD</t>
   </si>
   <si>
     <t>N° tabella -EFFORT -PROD</t>
+  </si>
+  <si>
+    <t>1000 (da cambiare)</t>
+  </si>
+  <si>
+    <t>Cod Parametro</t>
+  </si>
+  <si>
+    <t>* ( da implementare)</t>
+  </si>
+  <si>
+    <t>N° tabella - Piave -SVIL</t>
+  </si>
+  <si>
+    <t>N° tabella - Piave -PROD</t>
+  </si>
+  <si>
+    <t>N° tabella - X3Cloud (vecchio)</t>
+  </si>
+  <si>
+    <t>N° tabella - Terremerse - SVIL</t>
+  </si>
+  <si>
+    <t>N° tabella - Terremerse - COLL</t>
+  </si>
+  <si>
+    <t>N° tabella - Cloud 2024R2 v12 -TEST</t>
+  </si>
+  <si>
+    <t>* (da implementare)</t>
   </si>
 </sst>
 </file>
@@ -352,7 +367,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -365,8 +380,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -441,11 +468,75 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -481,9 +572,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -498,6 +586,49 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1892,7 +2023,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46.85546875" customWidth="1"/>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="44.140625" customWidth="1"/>
     <col min="3" max="3" width="169.85546875" customWidth="1"/>
     <col min="4" max="4" width="73.5703125" customWidth="1"/>
   </cols>
@@ -2004,7 +2135,7 @@
       <c r="A11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="16" t="s">
         <v>27</v>
       </c>
       <c r="C11" s="6"/>
@@ -2017,15 +2148,15 @@
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>47</v>
+      <c r="B13" s="16" t="s">
+        <v>43</v>
       </c>
       <c r="C13" s="6"/>
       <c r="D13" s="5">
@@ -2036,8 +2167,8 @@
       <c r="A14" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="18" t="s">
-        <v>48</v>
+      <c r="B14" s="17" t="s">
+        <v>44</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -2053,34 +2184,36 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29" customWidth="1"/>
+    <col min="1" max="1" width="37" customWidth="1"/>
     <col min="2" max="3" width="17.140625" customWidth="1"/>
     <col min="4" max="4" width="13.28515625" customWidth="1"/>
     <col min="5" max="5" width="28.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="15" t="s">
-        <v>51</v>
+      <c r="G2" s="14" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -2093,7 +2226,7 @@
       <c r="C3" s="10">
         <v>6911</v>
       </c>
-      <c r="D3" s="16"/>
+      <c r="D3" s="15"/>
       <c r="E3" s="10">
         <v>6205</v>
       </c>
@@ -2112,63 +2245,226 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FFEF73B-2A28-4DAD-A3A0-1A812F223D15}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.7109375" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="20.140625" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="3" max="3" width="4.140625" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="5" max="5" width="21.28515625" customWidth="1"/>
+    <col min="6" max="6" width="3.7109375" customWidth="1"/>
     <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" customWidth="1"/>
+    <col min="9" max="9" width="3.7109375" customWidth="1"/>
+    <col min="10" max="10" width="19.28515625" customWidth="1"/>
+    <col min="11" max="11" width="17" customWidth="1"/>
+    <col min="12" max="12" width="7" customWidth="1"/>
+    <col min="13" max="13" width="18.42578125" customWidth="1"/>
+    <col min="14" max="14" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:14" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="18"/>
+      <c r="D1" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" s="18"/>
+      <c r="G1" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" s="18"/>
+      <c r="J1" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="L1" s="18"/>
+      <c r="M1" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G1" s="15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="N1" s="34" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="25"/>
+      <c r="B2" s="25"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="20"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="20"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="20"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="10" t="s">
+      <c r="B3" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="F3" s="10">
-        <v>1000</v>
-      </c>
-      <c r="G3">
-        <v>1000</v>
-      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="29"/>
+      <c r="G3" s="33">
+        <v>6002</v>
+      </c>
+      <c r="H3" s="36">
+        <v>6002</v>
+      </c>
+      <c r="I3" s="30"/>
+      <c r="J3" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="K3" s="22">
+        <v>6002</v>
+      </c>
+      <c r="L3" s="10"/>
+      <c r="M3" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="N3" s="32" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="25"/>
+      <c r="B4" s="25"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="20"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="20"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="20"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="25"/>
+      <c r="B5" s="25"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="20"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="20"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="20"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="25"/>
+      <c r="B6" s="25"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="20"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="20"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="20"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="25"/>
+      <c r="B7" s="25"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="20"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="20"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="20"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="25"/>
+      <c r="B8" s="25"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="20"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="20"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="20"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="25"/>
+      <c r="B9" s="25"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="20"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="20"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="20"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="25"/>
+      <c r="B10" s="25"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="20"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="20"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="20"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="25"/>
+      <c r="B11" s="25"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="20"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="20"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="20"/>
+    </row>
+    <row r="12" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="27"/>
+      <c r="B12" s="27"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="24"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="24"/>
+      <c r="M12" s="23"/>
+      <c r="N12" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2179,7 +2475,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76CC19D8-B440-47A0-BCD1-D33842864B68}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
20° commit- aggiornamenti a livello di modulo patch
</commit_message>
<xml_diff>
--- a/patch/docs/patchList_protocolCore.xlsx
+++ b/patch/docs/patchList_protocolCore.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcorbara\Documents\ArgoX3_API_Mobile_CORE\patch\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5862CE6-9B47-45FB-8D1D-FCFA1A5BA9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D039F15-7993-46A1-AFBA-081149B68103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core - patchList" sheetId="1" r:id="rId1"/>
@@ -29,15 +29,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
   <si>
     <t>Data</t>
   </si>
   <si>
     <t>Nome Patch (Core)</t>
-  </si>
-  <si>
-    <t>Patch per  script core</t>
   </si>
   <si>
     <t>Elemento X3</t>
@@ -136,9 +133,6 @@
     <t>Pool SOAP</t>
   </si>
   <si>
-    <t>/</t>
-  </si>
-  <si>
     <t>AX3M_API_PROD ( non più Prod)</t>
   </si>
   <si>
@@ -173,9 +167,6 @@
   </si>
   <si>
     <t>N° tabella -EFFORT -TEST</t>
-  </si>
-  <si>
-    <t>Tabella Diversa - Controller (*Definizione- *Dati)</t>
   </si>
   <si>
     <t>YTDMENAX3M</t>
@@ -400,12 +391,99 @@
   <si>
     <t>N° parametro -EFFORT -PROD</t>
   </si>
+  <si>
+    <t>SRC_X3_V12_X_CORE_V1_2</t>
+  </si>
+  <si>
+    <t>26.02.2026</t>
+  </si>
+  <si>
+    <t>Patch per  script core (.src)</t>
+  </si>
+  <si>
+    <t>SRC_X3_V12_X_TRTC_V1_2</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nota</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: il capitolo  potrà variare in base all'ambiente e al dossier.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Tabella Diversa - Controller (*Definizione- *Dati)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nota</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: il N°  Tabella  potrà variare in base all'ambiente e al dossier.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">YTDMENAX3M - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nota</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: il valore del parametro generale  sarà uguale alla tabella diversa soprastante, dunque  potrà variare in base all'ambiente e al dossier.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,6 +512,12 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -614,7 +698,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -647,9 +731,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -661,9 +742,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -695,7 +773,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -743,11 +820,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2107,22 +2182,34 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>22</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="D1" s="47"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" t="s">
+        <v>65</v>
+      </c>
       <c r="C2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="32"/>
+        <v>20</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" t="s">
+        <v>65</v>
+      </c>
       <c r="C3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="32"/>
+        <v>66</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2140,29 +2227,29 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="135" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -2170,10 +2257,10 @@
     </row>
     <row r="4" spans="1:5" ht="173.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
@@ -2181,10 +2268,10 @@
     </row>
     <row r="5" spans="1:5" ht="260.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
@@ -2192,10 +2279,10 @@
     </row>
     <row r="6" spans="1:5" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
@@ -2203,10 +2290,10 @@
     </row>
     <row r="7" spans="1:5" ht="228" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
@@ -2214,64 +2301,64 @@
     </row>
     <row r="8" spans="1:5" ht="277.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
     </row>
     <row r="9" spans="1:5" ht="335.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>26</v>
+        <v>15</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>68</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="129.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="342" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="16" t="s">
         <v>24</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>23</v>
       </c>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
     </row>
     <row r="12" spans="1:5" ht="316.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>39</v>
+        <v>32</v>
+      </c>
+      <c r="B13" s="48" t="s">
+        <v>69</v>
       </c>
       <c r="C13" s="6"/>
       <c r="D13" s="5">
@@ -2280,17 +2367,18 @@
     </row>
     <row r="14" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>40</v>
+        <v>31</v>
+      </c>
+      <c r="B14" s="48" t="s">
+        <v>70</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2310,34 +2398,34 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="14" t="s">
+      <c r="A2" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>42</v>
+      <c r="F2" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" s="13" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" s="10">
         <v>6203</v>
@@ -2345,7 +2433,7 @@
       <c r="C3" s="10">
         <v>6911</v>
       </c>
-      <c r="D3" s="15"/>
+      <c r="D3" s="14"/>
       <c r="E3" s="10">
         <v>6205</v>
       </c>
@@ -2387,200 +2475,200 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="16"/>
+      <c r="D1" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="16"/>
+      <c r="G1" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" s="16"/>
+      <c r="J1" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="K1" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="30" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="F1" s="18"/>
-      <c r="G1" s="30" t="s">
-        <v>47</v>
-      </c>
-      <c r="H1" s="31" t="s">
-        <v>48</v>
-      </c>
-      <c r="I1" s="18"/>
-      <c r="J1" s="30" t="s">
+      <c r="L1" s="16"/>
+      <c r="M1" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="N1" s="28" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="18"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="18"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="18"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="18"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="10"/>
+      <c r="G3" s="19">
+        <v>6002</v>
+      </c>
+      <c r="H3" s="20">
+        <v>6002</v>
+      </c>
+      <c r="I3" s="10"/>
+      <c r="J3" s="19">
+        <v>6002</v>
+      </c>
+      <c r="K3" s="20">
+        <v>6002</v>
+      </c>
+      <c r="L3" s="10"/>
+      <c r="M3" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="N3" s="27" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="23"/>
+      <c r="B4" s="23"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="18"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="18"/>
+      <c r="J4" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="K1" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="L1" s="18"/>
-      <c r="M1" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="N1" s="30" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="20"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="20"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="20"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="20"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="21">
-        <v>6002</v>
-      </c>
-      <c r="H3" s="22">
-        <v>6002</v>
-      </c>
-      <c r="I3" s="10"/>
-      <c r="J3" s="21">
-        <v>6002</v>
-      </c>
-      <c r="K3" s="22">
-        <v>6002</v>
-      </c>
-      <c r="L3" s="10"/>
-      <c r="M3" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="N3" s="29" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="25"/>
-      <c r="B4" s="25"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="20"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="20"/>
-      <c r="J4" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="K4" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="M4" s="19"/>
-      <c r="N4" s="20"/>
+      <c r="K4" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="M4" s="17"/>
+      <c r="N4" s="18"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="25"/>
-      <c r="B5" s="25"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="20"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="20"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="20"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="20"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="23"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="18"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="18"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="18"/>
+      <c r="M5" s="17"/>
+      <c r="N5" s="18"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="25"/>
-      <c r="B6" s="25"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="20"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="20"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="20"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="20"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="23"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="18"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="18"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="18"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="18"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="25"/>
-      <c r="B7" s="25"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="20"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="20"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="20"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="20"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="23"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="18"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="18"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="18"/>
+      <c r="M7" s="17"/>
+      <c r="N7" s="18"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="25"/>
-      <c r="B8" s="25"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="20"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="20"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="20"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="20"/>
+      <c r="A8" s="23"/>
+      <c r="B8" s="23"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="18"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="18"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="18"/>
+      <c r="M8" s="17"/>
+      <c r="N8" s="18"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="25"/>
-      <c r="B9" s="25"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="20"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="20"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="20"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="20"/>
+      <c r="A9" s="23"/>
+      <c r="B9" s="23"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="18"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="18"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="18"/>
+      <c r="M9" s="17"/>
+      <c r="N9" s="18"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="25"/>
-      <c r="B10" s="25"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="20"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="20"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="20"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="20"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="23"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="18"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="18"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="18"/>
+      <c r="M10" s="17"/>
+      <c r="N10" s="18"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="25"/>
-      <c r="B11" s="25"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="20"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="20"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="20"/>
-      <c r="M11" s="19"/>
-      <c r="N11" s="20"/>
+      <c r="A11" s="23"/>
+      <c r="B11" s="23"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="18"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="18"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="18"/>
+      <c r="M11" s="17"/>
+      <c r="N11" s="18"/>
     </row>
     <row r="12" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="27"/>
-      <c r="B12" s="27"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="24"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="24"/>
-      <c r="J12" s="23"/>
-      <c r="K12" s="24"/>
-      <c r="M12" s="23"/>
-      <c r="N12" s="24"/>
+      <c r="A12" s="25"/>
+      <c r="B12" s="25"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="22"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="22"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="22"/>
+      <c r="M12" s="21"/>
+      <c r="N12" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2609,246 +2697,246 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="30" t="s">
+      <c r="A1" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="16"/>
+      <c r="E1" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="18"/>
-      <c r="E1" s="30" t="s">
+      <c r="G1" s="16"/>
+      <c r="H1" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="I1" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="30" t="s">
+      <c r="J1" s="16"/>
+      <c r="K1" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="18"/>
-      <c r="H1" s="30" t="s">
+      <c r="L1" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="I1" s="31" t="s">
+      <c r="M1" s="16"/>
+      <c r="N1" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="18"/>
-      <c r="K1" s="30" t="s">
+      <c r="O1" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="L1" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="M1" s="18"/>
-      <c r="N1" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="O1" s="30" t="s">
-        <v>66</v>
-      </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C2" s="25"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="20"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="20"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="20"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="20"/>
+      <c r="C2" s="23"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="18"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="18"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="18"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="18"/>
     </row>
     <row r="3" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="47" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="37"/>
-      <c r="E3" s="48" t="s">
-        <v>58</v>
-      </c>
-      <c r="F3" s="49" t="s">
-        <v>58</v>
-      </c>
-      <c r="G3" s="37"/>
-      <c r="H3" s="50">
+      <c r="A3" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="33"/>
+      <c r="C3" s="44" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="34"/>
+      <c r="E3" s="45" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="34"/>
+      <c r="H3" s="35">
         <v>6002</v>
       </c>
-      <c r="I3" s="51">
+      <c r="I3" s="36">
         <v>6002</v>
       </c>
-      <c r="J3" s="37"/>
-      <c r="K3" s="38">
+      <c r="J3" s="34"/>
+      <c r="K3" s="35">
         <v>6002</v>
       </c>
-      <c r="L3" s="39">
+      <c r="L3" s="36">
         <v>6002</v>
       </c>
-      <c r="M3" s="37"/>
-      <c r="N3" s="40" t="s">
-        <v>44</v>
-      </c>
-      <c r="O3" s="35" t="s">
-        <v>44</v>
+      <c r="M3" s="34"/>
+      <c r="N3" s="37" t="s">
+        <v>41</v>
+      </c>
+      <c r="O3" s="32" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="36"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="43"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="42" t="s">
-        <v>55</v>
-      </c>
-      <c r="L4" s="43" t="s">
-        <v>55</v>
-      </c>
-      <c r="M4" s="36"/>
-      <c r="N4" s="42"/>
-      <c r="O4" s="43"/>
+      <c r="A4" s="33"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="33"/>
+      <c r="K4" s="39" t="s">
+        <v>52</v>
+      </c>
+      <c r="L4" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="M4" s="33"/>
+      <c r="N4" s="39"/>
+      <c r="O4" s="40"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="36"/>
-      <c r="B5" s="36"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="43"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="42"/>
-      <c r="L5" s="43"/>
-      <c r="M5" s="36"/>
-      <c r="N5" s="42"/>
-      <c r="O5" s="43"/>
+      <c r="A5" s="33"/>
+      <c r="B5" s="33"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="39"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="33"/>
+      <c r="K5" s="39"/>
+      <c r="L5" s="40"/>
+      <c r="M5" s="33"/>
+      <c r="N5" s="39"/>
+      <c r="O5" s="40"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="36"/>
-      <c r="B6" s="36"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="43"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="42"/>
-      <c r="I6" s="43"/>
-      <c r="J6" s="36"/>
-      <c r="K6" s="42"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="36"/>
-      <c r="N6" s="42"/>
-      <c r="O6" s="43"/>
+      <c r="A6" s="33"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="39"/>
+      <c r="L6" s="40"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="39"/>
+      <c r="O6" s="40"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="36"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="42"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="43"/>
-      <c r="J7" s="36"/>
-      <c r="K7" s="42"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="36"/>
-      <c r="N7" s="42"/>
-      <c r="O7" s="43"/>
+      <c r="A7" s="33"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="39"/>
+      <c r="I7" s="40"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="39"/>
+      <c r="L7" s="40"/>
+      <c r="M7" s="33"/>
+      <c r="N7" s="39"/>
+      <c r="O7" s="40"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="36"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="42"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="36"/>
-      <c r="K8" s="42"/>
-      <c r="L8" s="43"/>
-      <c r="M8" s="36"/>
-      <c r="N8" s="42"/>
-      <c r="O8" s="43"/>
+      <c r="A8" s="33"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="40"/>
+      <c r="M8" s="33"/>
+      <c r="N8" s="39"/>
+      <c r="O8" s="40"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="36"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="42"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="42"/>
-      <c r="I9" s="43"/>
-      <c r="J9" s="36"/>
-      <c r="K9" s="42"/>
-      <c r="L9" s="43"/>
-      <c r="M9" s="36"/>
-      <c r="N9" s="42"/>
-      <c r="O9" s="43"/>
+      <c r="A9" s="33"/>
+      <c r="B9" s="33"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="40"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="39"/>
+      <c r="I9" s="40"/>
+      <c r="J9" s="33"/>
+      <c r="K9" s="39"/>
+      <c r="L9" s="40"/>
+      <c r="M9" s="33"/>
+      <c r="N9" s="39"/>
+      <c r="O9" s="40"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="36"/>
-      <c r="B10" s="36"/>
-      <c r="C10" s="41"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="42"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="42"/>
-      <c r="I10" s="43"/>
-      <c r="J10" s="36"/>
-      <c r="K10" s="42"/>
-      <c r="L10" s="43"/>
-      <c r="M10" s="36"/>
-      <c r="N10" s="42"/>
-      <c r="O10" s="43"/>
+      <c r="A10" s="33"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="40"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="39"/>
+      <c r="I10" s="40"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="39"/>
+      <c r="L10" s="40"/>
+      <c r="M10" s="33"/>
+      <c r="N10" s="39"/>
+      <c r="O10" s="40"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="36"/>
-      <c r="B11" s="36"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="43"/>
-      <c r="J11" s="36"/>
-      <c r="K11" s="42"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="36"/>
-      <c r="N11" s="42"/>
-      <c r="O11" s="43"/>
+      <c r="A11" s="33"/>
+      <c r="B11" s="33"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="39"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="39"/>
+      <c r="L11" s="40"/>
+      <c r="M11" s="33"/>
+      <c r="N11" s="39"/>
+      <c r="O11" s="40"/>
     </row>
     <row r="12" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="36"/>
-      <c r="B12" s="36"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="45"/>
-      <c r="I12" s="46"/>
-      <c r="J12" s="36"/>
-      <c r="K12" s="45"/>
-      <c r="L12" s="46"/>
-      <c r="M12" s="36"/>
-      <c r="N12" s="45"/>
-      <c r="O12" s="46"/>
+      <c r="A12" s="33"/>
+      <c r="B12" s="33"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="42"/>
+      <c r="I12" s="43"/>
+      <c r="J12" s="33"/>
+      <c r="K12" s="42"/>
+      <c r="L12" s="43"/>
+      <c r="M12" s="33"/>
+      <c r="N12" s="42"/>
+      <c r="O12" s="43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
22° commit: aggiornamento Git sezione Gestione patch e Tabelle Diverse
</commit_message>
<xml_diff>
--- a/patch/docs/patchList_protocolCore.xlsx
+++ b/patch/docs/patchList_protocolCore.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcorbara\Documents\ArgoX3_API_Mobile_CORE\patch\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D039F15-7993-46A1-AFBA-081149B68103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFDD7233-3E2F-43EE-9FE4-E99156A120CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core - patchList" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="76">
   <si>
     <t>Data</t>
   </si>
@@ -50,9 +50,6 @@
   </si>
   <si>
     <t xml:space="preserve">Descrizione Menù </t>
-  </si>
-  <si>
-    <t>* ArgoX3 Mobile - Lettura campo</t>
   </si>
   <si>
     <r>
@@ -108,9 +105,6 @@
   </si>
   <si>
     <t>Note-Descrizione</t>
-  </si>
-  <si>
-    <t>CHPT X3Cloud</t>
   </si>
   <si>
     <r>
@@ -478,6 +472,27 @@
       <t>: il valore del parametro generale  sarà uguale alla tabella diversa soprastante, dunque  potrà variare in base all'ambiente e al dossier.</t>
     </r>
   </si>
+  <si>
+    <t>CHPT Terremerse - PROD</t>
+  </si>
+  <si>
+    <t>da riportare qui</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ArgoX3 Mobile - Lettura campo</t>
+  </si>
+  <si>
+    <t>manca</t>
+  </si>
+  <si>
+    <t>CHPT X3Cloud (vecchio)</t>
+  </si>
+  <si>
+    <t>N° tabella - Terremerse - PROD</t>
+  </si>
+  <si>
+    <t>N° parametro - Terremerse - PROD</t>
+  </si>
 </sst>
 </file>
 
@@ -555,7 +570,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -694,11 +709,51 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -736,9 +791,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -761,20 +813,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -812,9 +856,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -823,6 +864,50 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2182,30 +2267,30 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" s="47"/>
+        <v>20</v>
+      </c>
+      <c r="D1" s="41"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2241,15 +2326,15 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="135" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -2257,10 +2342,10 @@
     </row>
     <row r="4" spans="1:5" ht="173.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
@@ -2268,10 +2353,10 @@
     </row>
     <row r="5" spans="1:5" ht="260.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
@@ -2279,10 +2364,10 @@
     </row>
     <row r="6" spans="1:5" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
@@ -2290,10 +2375,10 @@
     </row>
     <row r="7" spans="1:5" ht="228" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
@@ -2301,64 +2386,64 @@
     </row>
     <row r="8" spans="1:5" ht="277.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
     </row>
     <row r="9" spans="1:5" ht="335.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="129.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="342" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>21</v>
       </c>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
     </row>
     <row r="12" spans="1:5" ht="316.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="48" t="s">
-        <v>69</v>
+        <v>30</v>
+      </c>
+      <c r="B13" s="42" t="s">
+        <v>67</v>
       </c>
       <c r="C13" s="6"/>
       <c r="D13" s="5">
@@ -2367,10 +2452,10 @@
     </row>
     <row r="14" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" s="48" t="s">
-        <v>70</v>
+        <v>29</v>
+      </c>
+      <c r="B14" s="42" t="s">
+        <v>68</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -2384,68 +2469,167 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C911D19C-0B41-4FDE-964A-0EDA8C996211}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
-    <col min="2" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
     <col min="5" max="5" width="18.85546875" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="6" max="6" width="4.28515625" customWidth="1"/>
     <col min="7" max="7" width="19.28515625" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" customWidth="1"/>
+    <col min="8" max="8" width="3" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="3.7109375" customWidth="1"/>
+    <col min="12" max="12" width="15.5703125" customWidth="1"/>
+    <col min="13" max="13" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:13" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="25" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>27</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="C2" s="15"/>
       <c r="D2" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>50</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="15"/>
       <c r="G2" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="10">
+      <c r="H2" s="15"/>
+      <c r="I2" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="K2" s="15"/>
+      <c r="L2" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="23">
         <v>6203</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="10"/>
+      <c r="D3" s="18">
         <v>6911</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="10">
+      <c r="E3" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" s="10"/>
+      <c r="G3" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="H3" s="10"/>
+      <c r="I3" s="18">
         <v>6205</v>
       </c>
-      <c r="F3" s="10">
+      <c r="J3" s="19">
         <v>6205</v>
       </c>
-      <c r="G3" s="10">
+      <c r="K3" s="10"/>
+      <c r="L3" s="18">
         <v>6205</v>
       </c>
-      <c r="H3" s="10">
+      <c r="M3" s="19">
         <v>6205</v>
       </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="17"/>
+      <c r="G4" s="22"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="17"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="17"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="17"/>
+      <c r="G5" s="22"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="17"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="17"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="22"/>
+      <c r="B6" s="22"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="17"/>
+      <c r="G6" s="22"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="17"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="17"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="22"/>
+      <c r="B7" s="22"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="17"/>
+      <c r="G7" s="22"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="17"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="17"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="17"/>
+      <c r="G8" s="22"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="17"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="17"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="22"/>
+      <c r="B9" s="22"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="17"/>
+      <c r="G9" s="22"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="17"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="17"/>
+    </row>
+    <row r="10" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="21"/>
+      <c r="G10" s="24"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="21"/>
+      <c r="L10" s="20"/>
+      <c r="M10" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2455,220 +2639,237 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FFEF73B-2A28-4DAD-A3A0-1A812F223D15}">
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
     <col min="3" max="3" width="4.140625" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" customWidth="1"/>
-    <col min="5" max="5" width="21.28515625" customWidth="1"/>
-    <col min="6" max="6" width="3.7109375" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" customWidth="1"/>
+    <col min="7" max="7" width="3.28515625" customWidth="1"/>
     <col min="8" max="8" width="16.42578125" customWidth="1"/>
-    <col min="9" max="9" width="3.7109375" customWidth="1"/>
-    <col min="10" max="10" width="19.28515625" customWidth="1"/>
+    <col min="9" max="9" width="13.85546875" customWidth="1"/>
+    <col min="10" max="10" width="4.140625" customWidth="1"/>
     <col min="11" max="11" width="17" customWidth="1"/>
-    <col min="12" max="12" width="7" customWidth="1"/>
-    <col min="13" max="13" width="18.42578125" customWidth="1"/>
+    <col min="12" max="12" width="19.42578125" customWidth="1"/>
+    <col min="13" max="13" width="3.5703125" customWidth="1"/>
     <col min="14" max="14" width="19.140625" customWidth="1"/>
+    <col min="15" max="15" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:15" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="15"/>
+      <c r="D1" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="15"/>
+      <c r="H1" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="J1" s="15"/>
+      <c r="K1" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="L1" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="C1" s="16"/>
-      <c r="D1" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="E1" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="F1" s="16"/>
-      <c r="G1" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="H1" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="I1" s="16"/>
-      <c r="J1" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="K1" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="L1" s="16"/>
-      <c r="M1" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="N1" s="28" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="18"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="18"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="18"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="18"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
+      <c r="M1" s="15"/>
+      <c r="N1" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="19">
+      <c r="O1" s="25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="17"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="17"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="17"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="17"/>
+    </row>
+    <row r="3" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="48" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="49"/>
+      <c r="D3" s="50">
+        <v>6912</v>
+      </c>
+      <c r="E3" s="47" t="s">
+        <v>41</v>
+      </c>
+      <c r="F3" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="49"/>
+      <c r="H3" s="50">
         <v>6002</v>
       </c>
-      <c r="H3" s="20">
+      <c r="I3" s="51">
         <v>6002</v>
       </c>
-      <c r="I3" s="10"/>
-      <c r="J3" s="19">
+      <c r="J3" s="49"/>
+      <c r="K3" s="50">
         <v>6002</v>
       </c>
-      <c r="K3" s="20">
+      <c r="L3" s="51">
         <v>6002</v>
       </c>
-      <c r="L3" s="10"/>
-      <c r="M3" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="N3" s="27" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="18"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="18"/>
-      <c r="J4" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="K4" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="M4" s="17"/>
-      <c r="N4" s="18"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="23"/>
-      <c r="B5" s="23"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="18"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="18"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="18"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="18"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="23"/>
-      <c r="B6" s="23"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="18"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="18"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="18"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="18"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="23"/>
-      <c r="B7" s="23"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="18"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="18"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="18"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="18"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="23"/>
-      <c r="B8" s="23"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="18"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="18"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="18"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="18"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="23"/>
-      <c r="B9" s="23"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="18"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="18"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="18"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="18"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="18"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="18"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="18"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="18"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="23"/>
-      <c r="B11" s="23"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="18"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="18"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="18"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="18"/>
-    </row>
-    <row r="12" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="25"/>
-      <c r="B12" s="25"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="22"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="22"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="22"/>
-      <c r="M12" s="21"/>
-      <c r="N12" s="22"/>
+      <c r="M3" s="49"/>
+      <c r="N3" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" s="27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="17"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="17"/>
+      <c r="K4" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="N4" s="16"/>
+      <c r="O4" s="17"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="17"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="17"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="17"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="17"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="22"/>
+      <c r="B6" s="22"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="17"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="17"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="17"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="17"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="22"/>
+      <c r="B7" s="22"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="17"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="17"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="17"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="17"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="17"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="17"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="17"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="17"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="22"/>
+      <c r="B9" s="22"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="17"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="17"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="17"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="17"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="45"/>
+      <c r="F10" s="17"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="17"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="17"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="17"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="22"/>
+      <c r="B11" s="22"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="17"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="17"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="17"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="17"/>
+    </row>
+    <row r="12" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="21"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="21"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="21"/>
+      <c r="N12" s="20"/>
+      <c r="O12" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2677,266 +2878,284 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76CC19D8-B440-47A0-BCD1-D33842864B68}">
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="5.5703125" customWidth="1"/>
-    <col min="3" max="3" width="23.85546875" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="2.85546875" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.140625" customWidth="1"/>
-    <col min="5" max="5" width="18.85546875" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" customWidth="1"/>
-    <col min="7" max="7" width="4.42578125" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="3.28515625" customWidth="1"/>
     <col min="9" max="9" width="18.5703125" customWidth="1"/>
-    <col min="10" max="10" width="4.42578125" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.28515625" customWidth="1"/>
     <col min="12" max="12" width="19.5703125" customWidth="1"/>
-    <col min="14" max="14" width="18.140625" customWidth="1"/>
-    <col min="15" max="15" width="20.42578125" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" customWidth="1"/>
+    <col min="14" max="14" width="5.140625" customWidth="1"/>
+    <col min="15" max="15" width="14.7109375" customWidth="1"/>
+    <col min="16" max="16" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
-        <v>42</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="28" t="s">
+    <row r="1" spans="1:16" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="53" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="15"/>
+      <c r="E1" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D1" s="16"/>
-      <c r="E1" s="28" t="s">
+      <c r="F1" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="H1" s="15"/>
+      <c r="I1" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="28" t="s">
+      <c r="J1" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="G1" s="16"/>
-      <c r="H1" s="28" t="s">
+      <c r="K1" s="15"/>
+      <c r="L1" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="I1" s="29" t="s">
+      <c r="M1" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="28" t="s">
+      <c r="N1" s="15"/>
+      <c r="O1" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="L1" s="29" t="s">
+      <c r="P1" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="M1" s="16"/>
-      <c r="N1" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="O1" s="28" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C2" s="23"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="18"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="18"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="18"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="18"/>
-    </row>
-    <row r="3" spans="1:15" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="33" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="44" t="s">
-        <v>55</v>
-      </c>
-      <c r="D3" s="34"/>
-      <c r="E3" s="45" t="s">
-        <v>55</v>
-      </c>
-      <c r="F3" s="46" t="s">
-        <v>55</v>
-      </c>
-      <c r="G3" s="34"/>
-      <c r="H3" s="35">
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="C2" s="22"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="59"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="17"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="17"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="17"/>
+    </row>
+    <row r="3" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="28"/>
+      <c r="C3" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="29"/>
+      <c r="E3" s="44">
+        <v>6912</v>
+      </c>
+      <c r="F3" s="55" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" s="29"/>
+      <c r="I3" s="30">
         <v>6002</v>
       </c>
-      <c r="I3" s="36">
+      <c r="J3" s="31">
         <v>6002</v>
       </c>
-      <c r="J3" s="34"/>
-      <c r="K3" s="35">
+      <c r="K3" s="29"/>
+      <c r="L3" s="30">
         <v>6002</v>
       </c>
-      <c r="L3" s="36">
+      <c r="M3" s="31">
         <v>6002</v>
       </c>
-      <c r="M3" s="34"/>
-      <c r="N3" s="37" t="s">
-        <v>41</v>
-      </c>
+      <c r="N3" s="29"/>
       <c r="O3" s="32" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="33"/>
-      <c r="B4" s="33"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="40"/>
-      <c r="J4" s="33"/>
-      <c r="K4" s="39" t="s">
-        <v>52</v>
-      </c>
-      <c r="L4" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="M4" s="33"/>
-      <c r="N4" s="39"/>
-      <c r="O4" s="40"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="33"/>
-      <c r="B5" s="33"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="39"/>
-      <c r="I5" s="40"/>
-      <c r="J5" s="33"/>
-      <c r="K5" s="39"/>
-      <c r="L5" s="40"/>
-      <c r="M5" s="33"/>
-      <c r="N5" s="39"/>
-      <c r="O5" s="40"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="33"/>
-      <c r="B6" s="33"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="39"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="33"/>
-      <c r="K6" s="39"/>
-      <c r="L6" s="40"/>
-      <c r="M6" s="33"/>
-      <c r="N6" s="39"/>
-      <c r="O6" s="40"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="33"/>
-      <c r="B7" s="33"/>
-      <c r="C7" s="38"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="40"/>
-      <c r="J7" s="33"/>
-      <c r="K7" s="39"/>
-      <c r="L7" s="40"/>
-      <c r="M7" s="33"/>
-      <c r="N7" s="39"/>
-      <c r="O7" s="40"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="33"/>
-      <c r="B8" s="33"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="39"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="33"/>
-      <c r="K8" s="39"/>
-      <c r="L8" s="40"/>
-      <c r="M8" s="33"/>
-      <c r="N8" s="39"/>
-      <c r="O8" s="40"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="33"/>
-      <c r="B9" s="33"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="39"/>
-      <c r="I9" s="40"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="39"/>
-      <c r="L9" s="40"/>
-      <c r="M9" s="33"/>
-      <c r="N9" s="39"/>
-      <c r="O9" s="40"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="33"/>
-      <c r="B10" s="33"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="33"/>
-      <c r="K10" s="39"/>
-      <c r="L10" s="40"/>
-      <c r="M10" s="33"/>
-      <c r="N10" s="39"/>
-      <c r="O10" s="40"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="33"/>
-      <c r="B11" s="33"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="33"/>
-      <c r="H11" s="39"/>
-      <c r="I11" s="40"/>
-      <c r="J11" s="33"/>
-      <c r="K11" s="39"/>
-      <c r="L11" s="40"/>
-      <c r="M11" s="33"/>
-      <c r="N11" s="39"/>
-      <c r="O11" s="40"/>
-    </row>
-    <row r="12" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="33"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="42"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="33"/>
-      <c r="K12" s="42"/>
-      <c r="L12" s="43"/>
-      <c r="M12" s="33"/>
-      <c r="N12" s="42"/>
-      <c r="O12" s="43"/>
+        <v>39</v>
+      </c>
+      <c r="P3" s="27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="28"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="34"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="M4" s="35" t="s">
+        <v>50</v>
+      </c>
+      <c r="N4" s="28"/>
+      <c r="O4" s="34"/>
+      <c r="P4" s="35"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="34"/>
+      <c r="J5" s="35"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="34"/>
+      <c r="M5" s="35"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="34"/>
+      <c r="P5" s="35"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="28"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="56"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="28"/>
+      <c r="L6" s="34"/>
+      <c r="M6" s="35"/>
+      <c r="N6" s="28"/>
+      <c r="O6" s="34"/>
+      <c r="P6" s="35"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="28"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="56"/>
+      <c r="G7" s="35"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="35"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="35"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="34"/>
+      <c r="P7" s="35"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="28"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="56"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="35"/>
+      <c r="K8" s="28"/>
+      <c r="L8" s="34"/>
+      <c r="M8" s="35"/>
+      <c r="N8" s="28"/>
+      <c r="O8" s="34"/>
+      <c r="P8" s="35"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="28"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="35"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="35"/>
+      <c r="K9" s="28"/>
+      <c r="L9" s="34"/>
+      <c r="M9" s="35"/>
+      <c r="N9" s="28"/>
+      <c r="O9" s="34"/>
+      <c r="P9" s="35"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="35"/>
+      <c r="K10" s="28"/>
+      <c r="L10" s="34"/>
+      <c r="M10" s="35"/>
+      <c r="N10" s="28"/>
+      <c r="O10" s="34"/>
+      <c r="P10" s="35"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="56"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="35"/>
+      <c r="K11" s="28"/>
+      <c r="L11" s="34"/>
+      <c r="M11" s="35"/>
+      <c r="N11" s="28"/>
+      <c r="O11" s="34"/>
+      <c r="P11" s="35"/>
+    </row>
+    <row r="12" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="37"/>
+      <c r="F12" s="60"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="38"/>
+      <c r="K12" s="28"/>
+      <c r="L12" s="37"/>
+      <c r="M12" s="38"/>
+      <c r="N12" s="28"/>
+      <c r="O12" s="37"/>
+      <c r="P12" s="38"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Dettagli sulla gestione Patch AX3C
</commit_message>
<xml_diff>
--- a/patch/docs/patchList_protocolCore.xlsx
+++ b/patch/docs/patchList_protocolCore.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcorbara\Documents\ArgoX3_API_Mobile_CORE\patch\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{428BBDA4-7528-4839-9318-141A915C2964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD4F990C-B96E-4E02-B64B-34A4B73189C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Core - patchList" sheetId="1" r:id="rId1"/>
+    <sheet name="Core - patchList -Storico patch" sheetId="1" r:id="rId1"/>
     <sheet name="Core- elem porting manuale" sheetId="2" r:id="rId2"/>
     <sheet name="Menu" sheetId="3" r:id="rId3"/>
     <sheet name="Tabelle diverse" sheetId="4" r:id="rId4"/>
     <sheet name="Param Generali" sheetId="5" r:id="rId5"/>
+    <sheet name="Guida Inst elem manuali patch " sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="103">
   <si>
     <t>Nome Patch (Core)</t>
   </si>
@@ -563,6 +564,60 @@
   <si>
     <t>EFFORT (PROD)</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nota</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: il codice del menù local a cui è associato il campo  dipende dall'ambiente e progetto (l'esempio propone il menù locale di codice 6203)</t>
+    </r>
+  </si>
+  <si>
+    <t>Flussi</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>1-Installare Cod. Attività su  tutti gli ambienti di sviluppo coinvolti (YAX3C, YAX3M)</t>
+  </si>
+  <si>
+    <t>Ad es su :PROD e SVIL  o PROD &amp; TEST o PROD &amp; COLL</t>
+  </si>
+  <si>
+    <t>2- Riservare un capitolo unico (allineato) su  tutti gli ambienti di sviluppo coinvolti per i menù locali custom  ( ad es per il campo YSCANMODE)</t>
+  </si>
+  <si>
+    <t>3- inserire i campi custom Ax3m nelle Tab std</t>
+  </si>
+  <si>
+    <t>4- inserire i campi custom Ax3m nelle maschere std</t>
+  </si>
+  <si>
+    <t>5- Riservare un codice unico (allineato) su  tutti gli ambienti di sviluppo coinvolti perle tab diverse custom  ( ad es per la gestione del Menù funzioni)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 6- Definire il param generale associato alla Tab diversa (per gestione Menù funzioni Ax3m) su tutti gli ambienti di sviluppo coinvolti</t>
+  </si>
+  <si>
+    <t>da inserire</t>
+  </si>
 </sst>
 </file>
 
@@ -640,7 +695,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -819,18 +874,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -989,6 +1051,25 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1194,9 +1275,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>5876926</xdr:colOff>
+      <xdr:colOff>5033596</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>1493400</xdr:rowOff>
+      <xdr:rowOff>1286525</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1219,8 +1300,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5581651" y="4448176"/>
-          <a:ext cx="5505450" cy="1350524"/>
+          <a:off x="6438168" y="4905376"/>
+          <a:ext cx="4662120" cy="1143649"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1232,15 +1313,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>276226</xdr:colOff>
+      <xdr:colOff>239591</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>1740715</xdr:rowOff>
+      <xdr:rowOff>1337734</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>5876926</xdr:colOff>
+      <xdr:colOff>5840291</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>3010268</xdr:rowOff>
+      <xdr:rowOff>2607287</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1263,7 +1344,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5486401" y="6046015"/>
+          <a:off x="6306283" y="6100234"/>
           <a:ext cx="5600700" cy="1269553"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1584,15 +1665,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>8829675</xdr:colOff>
+      <xdr:colOff>5825637</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>257175</xdr:rowOff>
+      <xdr:rowOff>249848</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>11039712</xdr:colOff>
+      <xdr:colOff>8035674</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>4991100</xdr:rowOff>
+      <xdr:rowOff>4983773</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1615,7 +1696,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14039850" y="28879800"/>
+          <a:off x="11892329" y="32576233"/>
           <a:ext cx="2210037" cy="4733925"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1897,8 +1978,8 @@
       <xdr:rowOff>2761850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>8927328</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>669885</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>4134228</xdr:rowOff>
     </xdr:to>
@@ -2057,6 +2138,138 @@
         <a:xfrm>
           <a:off x="6332216" y="34137600"/>
           <a:ext cx="4361623" cy="1943988"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>219808</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>1626577</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2916116</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>2031989</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Immagine 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4EC281A8-DA04-C090-294B-188AA88F93C6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6286500" y="2014904"/>
+          <a:ext cx="2696308" cy="405412"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>366346</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>1795097</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3062654</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>2142559</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Immagine 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{671F41BB-1DFF-84D3-7E85-3843AB50498C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6433038" y="4330212"/>
+          <a:ext cx="2696308" cy="347462"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>322386</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2784231</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3575540</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>4089809</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Immagine 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDFA8F48-3883-091A-5A6D-B58C82ACBA4C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6389078" y="7546731"/>
+          <a:ext cx="3253154" cy="1305578"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2341,61 +2554,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="67" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="68" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="41"/>
+      <c r="D1" s="39"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="49" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="54" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="53" t="s">
+      <c r="C2" s="51" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="19" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="10"/>
+      <c r="B4" s="8"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="49" t="s">
         <v>77</v>
       </c>
-      <c r="B5" s="56" t="s">
+      <c r="B5" s="54" t="s">
         <v>75</v>
       </c>
-      <c r="C5" s="53" t="s">
+      <c r="C5" s="51" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="B6" s="57" t="s">
+      <c r="B6" s="55" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="19" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2412,21 +2625,21 @@
   <cols>
     <col min="1" max="1" width="46.85546875" customWidth="1"/>
     <col min="2" max="2" width="44.140625" customWidth="1"/>
-    <col min="3" max="3" width="169.85546875" customWidth="1"/>
+    <col min="3" max="3" width="123.85546875" customWidth="1"/>
     <col min="4" max="4" width="73.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="53" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2435,136 +2648,138 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:5" ht="168.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-    </row>
-    <row r="4" spans="1:5" ht="173.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="C3" s="4"/>
+      <c r="D3" s="40" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4" spans="1:5" ht="175.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-    </row>
-    <row r="5" spans="1:5" ht="260.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="C4" s="4"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="4"/>
+    </row>
+    <row r="5" spans="1:5" ht="330.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="4"/>
     </row>
     <row r="6" spans="1:5" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
     </row>
     <row r="7" spans="1:5" ht="228" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
     </row>
     <row r="8" spans="1:5" ht="277.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:5" ht="335.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="8" t="s">
+      <c r="C9" s="4"/>
+      <c r="D9" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="129.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="6" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="342" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
     </row>
     <row r="12" spans="1:5" ht="316.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="8" t="s">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="42" t="s">
+      <c r="B13" s="40" t="s">
         <v>60</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="5">
+      <c r="C13" s="4"/>
+      <c r="D13" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="42" t="s">
+      <c r="B14" s="40" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2599,195 +2814,199 @@
   <sheetData>
     <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:19" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="13" t="s">
+      <c r="C2" s="13"/>
+      <c r="D2" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="15"/>
-      <c r="G2" s="13" t="s">
+      <c r="F2" s="13"/>
+      <c r="G2" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="15"/>
-      <c r="I2" s="13" t="s">
+      <c r="H2" s="13"/>
+      <c r="I2" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="J2" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="K2" s="15"/>
-      <c r="L2" s="13" t="s">
+      <c r="K2" s="13"/>
+      <c r="L2" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="M2" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="P2" s="13" t="s">
+      <c r="P2" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="R2" s="13" t="s">
+      <c r="R2" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="S2" s="13" t="s">
+      <c r="S2" s="11" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="21">
         <v>6203</v>
       </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="18">
+      <c r="C3" s="8"/>
+      <c r="D3" s="16">
         <v>6911</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="43" t="s">
+      <c r="F3" s="8"/>
+      <c r="G3" s="41" t="s">
         <v>63</v>
       </c>
-      <c r="H3" s="10"/>
-      <c r="I3" s="18">
+      <c r="H3" s="8"/>
+      <c r="I3" s="16">
         <v>6205</v>
       </c>
-      <c r="J3" s="19">
+      <c r="J3" s="17">
         <v>6205</v>
       </c>
-      <c r="K3" s="10"/>
-      <c r="L3" s="18">
+      <c r="K3" s="8"/>
+      <c r="L3" s="16">
         <v>6205</v>
       </c>
-      <c r="M3" s="19">
+      <c r="M3" s="17">
         <v>6205</v>
       </c>
-      <c r="O3" s="47">
+      <c r="O3" s="45">
         <v>6990</v>
       </c>
-      <c r="P3" s="60" t="s">
+      <c r="P3" s="58" t="s">
         <v>81</v>
       </c>
-      <c r="R3" s="47"/>
-      <c r="S3" s="60"/>
+      <c r="R3" s="45">
+        <v>6900</v>
+      </c>
+      <c r="S3" s="58">
+        <v>6900</v>
+      </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" s="22"/>
-      <c r="B4" s="22"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="17"/>
-      <c r="G4" s="22"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="17"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="17"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="17"/>
-      <c r="R4" s="16"/>
-      <c r="S4" s="17"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="15"/>
+      <c r="G4" s="20"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="15"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="15"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="15"/>
+      <c r="R4" s="14"/>
+      <c r="S4" s="15"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A5" s="22"/>
-      <c r="B5" s="22"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="17"/>
-      <c r="G5" s="22"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="17"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="17"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="17"/>
-      <c r="R5" s="16"/>
-      <c r="S5" s="17"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="15"/>
+      <c r="G5" s="20"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="15"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="15"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="15"/>
+      <c r="R5" s="14"/>
+      <c r="S5" s="15"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" s="22"/>
-      <c r="B6" s="22"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="17"/>
-      <c r="G6" s="22"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="17"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="17"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="17"/>
-      <c r="R6" s="16"/>
-      <c r="S6" s="17"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="20"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="15"/>
+      <c r="G6" s="20"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="15"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="15"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="15"/>
+      <c r="R6" s="14"/>
+      <c r="S6" s="15"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" s="22"/>
-      <c r="B7" s="22"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="17"/>
-      <c r="G7" s="22"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="17"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="17"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="17"/>
-      <c r="R7" s="16"/>
-      <c r="S7" s="17"/>
+      <c r="A7" s="20"/>
+      <c r="B7" s="20"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="15"/>
+      <c r="G7" s="20"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="15"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="15"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="15"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="15"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A8" s="22"/>
-      <c r="B8" s="22"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="17"/>
-      <c r="G8" s="22"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="17"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="17"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="17"/>
-      <c r="R8" s="16"/>
-      <c r="S8" s="17"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="15"/>
+      <c r="G8" s="20"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="15"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="15"/>
+      <c r="O8" s="14"/>
+      <c r="P8" s="15"/>
+      <c r="R8" s="14"/>
+      <c r="S8" s="15"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A9" s="22"/>
-      <c r="B9" s="22"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="17"/>
-      <c r="G9" s="22"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="17"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="17"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="17"/>
-      <c r="R9" s="16"/>
-      <c r="S9" s="17"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="15"/>
+      <c r="G9" s="20"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="15"/>
+      <c r="L9" s="14"/>
+      <c r="M9" s="15"/>
+      <c r="O9" s="14"/>
+      <c r="P9" s="15"/>
+      <c r="R9" s="14"/>
+      <c r="S9" s="15"/>
     </row>
     <row r="10" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="21"/>
-      <c r="G10" s="24"/>
-      <c r="I10" s="20"/>
-      <c r="J10" s="21"/>
-      <c r="L10" s="20"/>
-      <c r="M10" s="21"/>
-      <c r="O10" s="20"/>
-      <c r="P10" s="21"/>
-      <c r="R10" s="20"/>
-      <c r="S10" s="21"/>
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="19"/>
+      <c r="G10" s="22"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="19"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="19"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="19"/>
+      <c r="R10" s="18"/>
+      <c r="S10" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2822,271 +3041,275 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="15"/>
-      <c r="D1" s="25" t="s">
+      <c r="C1" s="13"/>
+      <c r="D1" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="15"/>
-      <c r="H1" s="25" t="s">
+      <c r="G1" s="13"/>
+      <c r="H1" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="I1" s="26" t="s">
+      <c r="I1" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="J1" s="15"/>
-      <c r="K1" s="25" t="s">
+      <c r="J1" s="13"/>
+      <c r="K1" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="L1" s="26" t="s">
+      <c r="L1" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="15"/>
-      <c r="N1" s="25" t="s">
+      <c r="M1" s="13"/>
+      <c r="N1" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="O1" s="25" t="s">
+      <c r="O1" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="58" t="s">
+      <c r="Q1" s="56" t="s">
         <v>82</v>
       </c>
-      <c r="R1" s="25" t="s">
+      <c r="R1" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="T1" s="58" t="s">
+      <c r="T1" s="56" t="s">
         <v>86</v>
       </c>
-      <c r="U1" s="25" t="s">
+      <c r="U1" s="23" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A2" s="22"/>
-      <c r="B2" s="22"/>
-      <c r="D2" s="16"/>
-      <c r="F2" s="17"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="17"/>
-      <c r="K2" s="16"/>
-      <c r="L2" s="17"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="17"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="17"/>
-      <c r="T2" s="16"/>
-      <c r="U2" s="17"/>
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="D2" s="14"/>
+      <c r="F2" s="15"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="15"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="15"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="15"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="15"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="15"/>
     </row>
     <row r="3" spans="1:21" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="44" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="45"/>
-      <c r="D3" s="47">
+      <c r="C3" s="43"/>
+      <c r="D3" s="45">
         <v>6912</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="48" t="s">
+      <c r="F3" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="G3" s="45"/>
-      <c r="H3" s="47">
+      <c r="G3" s="43"/>
+      <c r="H3" s="45">
         <v>6002</v>
       </c>
-      <c r="I3" s="48">
+      <c r="I3" s="46">
         <v>6002</v>
       </c>
-      <c r="J3" s="45"/>
-      <c r="K3" s="47">
+      <c r="J3" s="43"/>
+      <c r="K3" s="45">
         <v>6003</v>
       </c>
-      <c r="L3" s="48">
+      <c r="L3" s="46">
         <v>6003</v>
       </c>
-      <c r="M3" s="45"/>
-      <c r="N3" s="49" t="s">
+      <c r="M3" s="43"/>
+      <c r="N3" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="O3" s="27" t="s">
+      <c r="O3" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="Q3" s="16">
+      <c r="Q3" s="14">
         <v>6990</v>
       </c>
-      <c r="R3" s="17">
+      <c r="R3" s="15">
         <v>6990</v>
       </c>
-      <c r="T3" s="16"/>
-      <c r="U3" s="17"/>
+      <c r="T3" s="14">
+        <v>6900</v>
+      </c>
+      <c r="U3" s="15">
+        <v>6900</v>
+      </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A4" s="22"/>
-      <c r="B4" s="22"/>
-      <c r="D4" s="16"/>
-      <c r="F4" s="17"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="17"/>
-      <c r="K4" s="16" t="s">
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
+      <c r="D4" s="14"/>
+      <c r="F4" s="15"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="15"/>
+      <c r="K4" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="L4" s="17" t="s">
+      <c r="L4" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="N4" s="16"/>
-      <c r="O4" s="17"/>
-      <c r="Q4" s="16" t="s">
+      <c r="N4" s="14"/>
+      <c r="O4" s="15"/>
+      <c r="Q4" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="R4" s="17" t="s">
+      <c r="R4" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="T4" s="16"/>
-      <c r="U4" s="17"/>
+      <c r="T4" s="14"/>
+      <c r="U4" s="15"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A5" s="22"/>
-      <c r="B5" s="22"/>
-      <c r="D5" s="16"/>
-      <c r="F5" s="17"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="17"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="17"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="17"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="17"/>
-      <c r="T5" s="16"/>
-      <c r="U5" s="17"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
+      <c r="D5" s="14"/>
+      <c r="F5" s="15"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="15"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="15"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="15"/>
+      <c r="Q5" s="14"/>
+      <c r="R5" s="15"/>
+      <c r="T5" s="14"/>
+      <c r="U5" s="15"/>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A6" s="22"/>
-      <c r="B6" s="22"/>
-      <c r="D6" s="16"/>
-      <c r="F6" s="17"/>
-      <c r="H6" s="16"/>
-      <c r="I6" s="17"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="17"/>
-      <c r="N6" s="16"/>
-      <c r="O6" s="17"/>
-      <c r="Q6" s="16"/>
-      <c r="R6" s="17"/>
-      <c r="T6" s="16"/>
-      <c r="U6" s="17"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="20"/>
+      <c r="D6" s="14"/>
+      <c r="F6" s="15"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="15"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="15"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="15"/>
+      <c r="Q6" s="14"/>
+      <c r="R6" s="15"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="15"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A7" s="22"/>
-      <c r="B7" s="22"/>
-      <c r="D7" s="16"/>
-      <c r="F7" s="17"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="17"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="17"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="17"/>
-      <c r="Q7" s="16"/>
-      <c r="R7" s="17"/>
-      <c r="T7" s="16"/>
-      <c r="U7" s="17"/>
+      <c r="A7" s="20"/>
+      <c r="B7" s="20"/>
+      <c r="D7" s="14"/>
+      <c r="F7" s="15"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="15"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="15"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="15"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="15"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="15"/>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A8" s="22"/>
-      <c r="B8" s="22"/>
-      <c r="D8" s="16"/>
-      <c r="F8" s="17"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="17"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="17"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="17"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="17"/>
-      <c r="T8" s="16"/>
-      <c r="U8" s="17"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="D8" s="14"/>
+      <c r="F8" s="15"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="15"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="15"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="15"/>
+      <c r="Q8" s="14"/>
+      <c r="R8" s="15"/>
+      <c r="T8" s="14"/>
+      <c r="U8" s="15"/>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A9" s="22"/>
-      <c r="B9" s="22"/>
-      <c r="D9" s="16"/>
-      <c r="F9" s="17"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="17"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="17"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="17"/>
-      <c r="Q9" s="16"/>
-      <c r="R9" s="17"/>
-      <c r="T9" s="16"/>
-      <c r="U9" s="17"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="D9" s="14"/>
+      <c r="F9" s="15"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="15"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="15"/>
+      <c r="N9" s="14"/>
+      <c r="O9" s="15"/>
+      <c r="Q9" s="14"/>
+      <c r="R9" s="15"/>
+      <c r="T9" s="14"/>
+      <c r="U9" s="15"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A10" s="22"/>
-      <c r="B10" s="22"/>
-      <c r="D10" s="16"/>
-      <c r="F10" s="17"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="17"/>
-      <c r="K10" s="16"/>
-      <c r="L10" s="17"/>
-      <c r="N10" s="16"/>
-      <c r="O10" s="17"/>
-      <c r="Q10" s="16"/>
-      <c r="R10" s="17"/>
-      <c r="T10" s="16"/>
-      <c r="U10" s="17"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="D10" s="14"/>
+      <c r="F10" s="15"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="15"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="15"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="15"/>
+      <c r="Q10" s="14"/>
+      <c r="R10" s="15"/>
+      <c r="T10" s="14"/>
+      <c r="U10" s="15"/>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A11" s="22"/>
-      <c r="B11" s="22"/>
-      <c r="D11" s="16"/>
-      <c r="F11" s="17"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="17"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="17"/>
-      <c r="N11" s="16"/>
-      <c r="O11" s="17"/>
-      <c r="Q11" s="16"/>
-      <c r="R11" s="17"/>
-      <c r="T11" s="16"/>
-      <c r="U11" s="17"/>
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="D11" s="14"/>
+      <c r="F11" s="15"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="15"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="15"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="15"/>
+      <c r="Q11" s="14"/>
+      <c r="R11" s="15"/>
+      <c r="T11" s="14"/>
+      <c r="U11" s="15"/>
     </row>
     <row r="12" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="24"/>
-      <c r="B12" s="24"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="21"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="21"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="21"/>
-      <c r="N12" s="20"/>
-      <c r="O12" s="21"/>
-      <c r="Q12" s="20"/>
-      <c r="R12" s="21"/>
-      <c r="T12" s="20"/>
-      <c r="U12" s="21"/>
+      <c r="A12" s="22"/>
+      <c r="B12" s="22"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="19"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="19"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="19"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="19"/>
+      <c r="Q12" s="18"/>
+      <c r="R12" s="19"/>
+      <c r="T12" s="18"/>
+      <c r="U12" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3119,331 +3342,445 @@
     <col min="19" max="19" width="14.28515625" customWidth="1"/>
     <col min="20" max="20" width="3.85546875" customWidth="1"/>
     <col min="21" max="21" width="10.28515625" customWidth="1"/>
+    <col min="22" max="22" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="61" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="25" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="15"/>
-      <c r="E1" s="25" t="s">
+      <c r="D1" s="13"/>
+      <c r="E1" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="H1" s="15"/>
-      <c r="I1" s="25" t="s">
+      <c r="H1" s="13"/>
+      <c r="I1" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="J1" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="K1" s="15"/>
-      <c r="L1" s="25" t="s">
+      <c r="K1" s="13"/>
+      <c r="L1" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="M1" s="26" t="s">
+      <c r="M1" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="N1" s="15"/>
-      <c r="O1" s="25" t="s">
+      <c r="N1" s="13"/>
+      <c r="O1" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="P1" s="25" t="s">
+      <c r="P1" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="58" t="s">
+      <c r="Q1" s="27"/>
+      <c r="R1" s="56" t="s">
         <v>79</v>
       </c>
-      <c r="S1" s="25" t="s">
+      <c r="S1" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="T1" s="29"/>
-      <c r="U1" s="58" t="s">
+      <c r="T1" s="27"/>
+      <c r="U1" s="56" t="s">
         <v>86</v>
       </c>
-      <c r="V1" s="25" t="s">
+      <c r="V1" s="23" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="C2" s="22"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="53"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="17"/>
-      <c r="L2" s="16"/>
-      <c r="M2" s="17"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="17"/>
-      <c r="R2" s="59"/>
-      <c r="S2" s="60"/>
-      <c r="U2" s="16"/>
-      <c r="V2" s="17"/>
+      <c r="C2" s="20"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="51"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="15"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="15"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="15"/>
+      <c r="R2" s="57"/>
+      <c r="S2" s="58"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="15"/>
     </row>
     <row r="3" spans="1:22" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="39" t="s">
+      <c r="B3" s="26"/>
+      <c r="C3" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30">
+      <c r="D3" s="27"/>
+      <c r="E3" s="28">
         <v>6912</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="48" t="s">
         <v>46</v>
       </c>
-      <c r="G3" s="40" t="s">
+      <c r="G3" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="H3" s="29"/>
-      <c r="I3" s="30">
+      <c r="H3" s="27"/>
+      <c r="I3" s="28">
         <v>6002</v>
       </c>
-      <c r="J3" s="31">
+      <c r="J3" s="29">
         <v>6002</v>
       </c>
-      <c r="K3" s="29"/>
-      <c r="L3" s="30">
+      <c r="K3" s="27"/>
+      <c r="L3" s="28">
         <v>6002</v>
       </c>
-      <c r="M3" s="31">
+      <c r="M3" s="29">
         <v>6002</v>
       </c>
-      <c r="N3" s="29"/>
-      <c r="O3" s="32" t="s">
+      <c r="N3" s="27"/>
+      <c r="O3" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="P3" s="27" t="s">
+      <c r="P3" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="R3" s="59">
+      <c r="R3" s="57">
         <v>6990</v>
       </c>
-      <c r="S3" s="60">
+      <c r="S3" s="58">
         <v>6990</v>
       </c>
-      <c r="U3" s="16"/>
-      <c r="V3" s="17"/>
+      <c r="U3" s="14">
+        <v>6900</v>
+      </c>
+      <c r="V3" s="15" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="4" spans="1:22" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="28"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="35"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="34" t="s">
+      <c r="A4" s="26"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="33"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="M4" s="35" t="s">
+      <c r="M4" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="N4" s="28"/>
-      <c r="O4" s="34"/>
-      <c r="P4" s="35"/>
-      <c r="R4" s="59" t="s">
+      <c r="N4" s="26"/>
+      <c r="O4" s="32"/>
+      <c r="P4" s="33"/>
+      <c r="R4" s="57" t="s">
         <v>85</v>
       </c>
-      <c r="S4" s="60" t="s">
+      <c r="S4" s="58" t="s">
         <v>85</v>
       </c>
-      <c r="U4" s="16"/>
-      <c r="V4" s="17"/>
+      <c r="U4" s="14"/>
+      <c r="V4" s="15"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A5" s="28"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="35"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="35"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="35"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="34"/>
-      <c r="P5" s="35"/>
-      <c r="R5" s="59"/>
-      <c r="S5" s="60"/>
-      <c r="U5" s="16"/>
-      <c r="V5" s="17"/>
+      <c r="A5" s="26"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="33"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="33"/>
+      <c r="N5" s="26"/>
+      <c r="O5" s="32"/>
+      <c r="P5" s="33"/>
+      <c r="R5" s="57"/>
+      <c r="S5" s="58"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="15"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A6" s="28"/>
-      <c r="B6" s="28"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="28"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="35"/>
-      <c r="K6" s="28"/>
-      <c r="L6" s="34"/>
-      <c r="M6" s="35"/>
-      <c r="N6" s="28"/>
-      <c r="O6" s="34"/>
-      <c r="P6" s="35"/>
-      <c r="R6" s="59"/>
-      <c r="S6" s="60"/>
-      <c r="U6" s="16"/>
-      <c r="V6" s="17"/>
+      <c r="A6" s="26"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="33"/>
+      <c r="R6" s="57"/>
+      <c r="S6" s="58"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="15"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A7" s="28"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="35"/>
-      <c r="K7" s="28"/>
-      <c r="L7" s="34"/>
-      <c r="M7" s="35"/>
-      <c r="N7" s="28"/>
-      <c r="O7" s="34"/>
-      <c r="P7" s="35"/>
-      <c r="R7" s="59"/>
-      <c r="S7" s="60"/>
-      <c r="U7" s="16"/>
-      <c r="V7" s="17"/>
+      <c r="A7" s="26"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="32"/>
+      <c r="M7" s="33"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="32"/>
+      <c r="P7" s="33"/>
+      <c r="R7" s="57"/>
+      <c r="S7" s="58"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="15"/>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A8" s="28"/>
-      <c r="B8" s="28"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="34"/>
-      <c r="J8" s="35"/>
-      <c r="K8" s="28"/>
-      <c r="L8" s="34"/>
-      <c r="M8" s="35"/>
-      <c r="N8" s="28"/>
-      <c r="O8" s="34"/>
-      <c r="P8" s="35"/>
-      <c r="R8" s="59"/>
-      <c r="S8" s="60"/>
-      <c r="U8" s="16"/>
-      <c r="V8" s="17"/>
+      <c r="A8" s="26"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="32"/>
+      <c r="M8" s="33"/>
+      <c r="N8" s="26"/>
+      <c r="O8" s="32"/>
+      <c r="P8" s="33"/>
+      <c r="R8" s="57"/>
+      <c r="S8" s="58"/>
+      <c r="U8" s="14"/>
+      <c r="V8" s="15"/>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A9" s="28"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="28"/>
-      <c r="L9" s="34"/>
-      <c r="M9" s="35"/>
-      <c r="N9" s="28"/>
-      <c r="O9" s="34"/>
-      <c r="P9" s="35"/>
-      <c r="R9" s="59"/>
-      <c r="S9" s="60"/>
-      <c r="U9" s="16"/>
-      <c r="V9" s="17"/>
+      <c r="A9" s="26"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="33"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="32"/>
+      <c r="M9" s="33"/>
+      <c r="N9" s="26"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="33"/>
+      <c r="R9" s="57"/>
+      <c r="S9" s="58"/>
+      <c r="U9" s="14"/>
+      <c r="V9" s="15"/>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A10" s="28"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="34"/>
-      <c r="M10" s="35"/>
-      <c r="N10" s="28"/>
-      <c r="O10" s="34"/>
-      <c r="P10" s="35"/>
-      <c r="R10" s="59"/>
-      <c r="S10" s="60"/>
-      <c r="U10" s="16"/>
-      <c r="V10" s="17"/>
+      <c r="A10" s="26"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="26"/>
+      <c r="L10" s="32"/>
+      <c r="M10" s="33"/>
+      <c r="N10" s="26"/>
+      <c r="O10" s="32"/>
+      <c r="P10" s="33"/>
+      <c r="R10" s="57"/>
+      <c r="S10" s="58"/>
+      <c r="U10" s="14"/>
+      <c r="V10" s="15"/>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A11" s="28"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="35"/>
-      <c r="K11" s="28"/>
-      <c r="L11" s="34"/>
-      <c r="M11" s="35"/>
-      <c r="N11" s="28"/>
-      <c r="O11" s="34"/>
-      <c r="P11" s="35"/>
-      <c r="R11" s="59"/>
-      <c r="S11" s="60"/>
-      <c r="U11" s="16"/>
-      <c r="V11" s="17"/>
+      <c r="A11" s="26"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="26"/>
+      <c r="L11" s="32"/>
+      <c r="M11" s="33"/>
+      <c r="N11" s="26"/>
+      <c r="O11" s="32"/>
+      <c r="P11" s="33"/>
+      <c r="R11" s="57"/>
+      <c r="S11" s="58"/>
+      <c r="U11" s="14"/>
+      <c r="V11" s="15"/>
     </row>
     <row r="12" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="28"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="36"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="54"/>
-      <c r="G12" s="38"/>
-      <c r="H12" s="28"/>
-      <c r="I12" s="37"/>
-      <c r="J12" s="38"/>
-      <c r="K12" s="28"/>
-      <c r="L12" s="37"/>
-      <c r="M12" s="38"/>
-      <c r="N12" s="28"/>
-      <c r="O12" s="37"/>
-      <c r="P12" s="38"/>
-      <c r="R12" s="61"/>
-      <c r="S12" s="62"/>
-      <c r="U12" s="20"/>
-      <c r="V12" s="21"/>
+      <c r="A12" s="26"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="35"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="26"/>
+      <c r="L12" s="35"/>
+      <c r="M12" s="36"/>
+      <c r="N12" s="26"/>
+      <c r="O12" s="35"/>
+      <c r="P12" s="36"/>
+      <c r="R12" s="59"/>
+      <c r="S12" s="60"/>
+      <c r="U12" s="18"/>
+      <c r="V12" s="19"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F716B07-04C2-48BB-91BF-B7D324A59533}">
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="99" customWidth="1"/>
+    <col min="2" max="2" width="96.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="66" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="62"/>
+    </row>
+    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="64" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" s="58" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="64" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="58"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="64" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" s="58"/>
+    </row>
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="64" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" s="58" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="64" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="58" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="64"/>
+      <c r="B9" s="58"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="64"/>
+      <c r="B10" s="58"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="64"/>
+      <c r="B11" s="58"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="64"/>
+      <c r="B12" s="58"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="64"/>
+      <c r="B13" s="58"/>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="64"/>
+      <c r="B14" s="58"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="64"/>
+      <c r="B15" s="58"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="64"/>
+      <c r="B16" s="58"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="64"/>
+      <c r="B17" s="58"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="64"/>
+      <c r="B18" s="58"/>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="65"/>
+      <c r="B19" s="60"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>